<commit_message>
update rCNV annotation from clinicalgenome website
</commit_message>
<xml_diff>
--- a/resources/rCNV/docs/frequency_comparison.xlsx
+++ b/resources/rCNV/docs/frequency_comparison.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -1171,37 +1171,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1275,7 +1275,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K244"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="33.15"/>
@@ -1310,7 +1310,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="17.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -5472,8 +5472,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>